<commit_message>
updated manual and working technical bot
</commit_message>
<xml_diff>
--- a/Lakshmi.xlsx
+++ b/Lakshmi.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H452"/>
+  <dimension ref="A1:H564"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="24.33203125" customWidth="1" style="1" min="1" max="1"/>
@@ -14037,6 +14037,2694 @@
       </c>
       <c r="F452" t="n">
         <v>676</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2026-01-27 10:35:03</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>NIFTY2620324650PE</t>
+        </is>
+      </c>
+      <c r="C453" t="n">
+        <v>107.15</v>
+      </c>
+      <c r="D453" t="n">
+        <v>100.55</v>
+      </c>
+      <c r="E453" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F453" t="n">
+        <v>-6864</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2026-01-27 10:40:17</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>NIFTY2620324650PE</t>
+        </is>
+      </c>
+      <c r="C454" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="D454" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="E454" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F454" t="n">
+        <v>1144</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2026-01-27 10:41:47</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>NIFTY2620324650PE</t>
+        </is>
+      </c>
+      <c r="C455" t="n">
+        <v>111.15</v>
+      </c>
+      <c r="D455" t="n">
+        <v>111.15</v>
+      </c>
+      <c r="E455" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F455" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2026-01-27 10:46:56</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>NIFTY2620325600CE</t>
+        </is>
+      </c>
+      <c r="C456" t="n">
+        <v>101.85</v>
+      </c>
+      <c r="D456" t="n">
+        <v>101.65</v>
+      </c>
+      <c r="E456" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F456" t="n">
+        <v>-208</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026-01-27 11:02:54</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>NIFTY2620325600CE</t>
+        </is>
+      </c>
+      <c r="C457" t="n">
+        <v>97.3</v>
+      </c>
+      <c r="D457" t="n">
+        <v>97.09999999999999</v>
+      </c>
+      <c r="E457" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F457" t="n">
+        <v>-208</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026-01-27 11:04:41</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>NIFTY2620325550CE</t>
+        </is>
+      </c>
+      <c r="C458" t="n">
+        <v>110.15</v>
+      </c>
+      <c r="D458" t="n">
+        <v>111.1</v>
+      </c>
+      <c r="E458" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F458" t="n">
+        <v>988</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>2026-01-27 11:08:10</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>NIFTY2620325550CE</t>
+        </is>
+      </c>
+      <c r="C459" t="n">
+        <v>110.75</v>
+      </c>
+      <c r="D459" t="n">
+        <v>109.3</v>
+      </c>
+      <c r="E459" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F459" t="n">
+        <v>-1508</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026-01-27 11:09:40</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>NIFTY2620325550CE</t>
+        </is>
+      </c>
+      <c r="C460" t="n">
+        <v>113.25</v>
+      </c>
+      <c r="D460" t="n">
+        <v>118</v>
+      </c>
+      <c r="E460" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F460" t="n">
+        <v>4940</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026-01-27 11:12:42</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>NIFTY2620325650CE</t>
+        </is>
+      </c>
+      <c r="C461" t="n">
+        <v>89.40000000000001</v>
+      </c>
+      <c r="D461" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="E461" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F461" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026-01-28 11:35:54</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>NIFTY2620325050PE</t>
+        </is>
+      </c>
+      <c r="C462" t="n">
+        <v>105.95</v>
+      </c>
+      <c r="D462" t="n">
+        <v>106.15</v>
+      </c>
+      <c r="E462" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F462" t="n">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-01-28 11:38:19</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>NIFTY2620325050PE</t>
+        </is>
+      </c>
+      <c r="C463" t="n">
+        <v>107.7</v>
+      </c>
+      <c r="D463" t="n">
+        <v>111.45</v>
+      </c>
+      <c r="E463" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F463" t="n">
+        <v>3900</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-01-28 11:45:20</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>NIFTY2620325000PE</t>
+        </is>
+      </c>
+      <c r="C464" t="n">
+        <v>103.45</v>
+      </c>
+      <c r="D464" t="n">
+        <v>104.2</v>
+      </c>
+      <c r="E464" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F464" t="n">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026-01-28 11:52:02</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>NIFTY2620325650CE</t>
+        </is>
+      </c>
+      <c r="C465" t="n">
+        <v>100.2</v>
+      </c>
+      <c r="D465" t="n">
+        <v>100.8</v>
+      </c>
+      <c r="E465" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F465" t="n">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-01-28 12:01:36</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>NIFTY2620325650CE</t>
+        </is>
+      </c>
+      <c r="C466" t="n">
+        <v>100.15</v>
+      </c>
+      <c r="D466" t="n">
+        <v>101</v>
+      </c>
+      <c r="E466" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F466" t="n">
+        <v>884</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-01-28 12:07:12</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>NIFTY2620325650CE</t>
+        </is>
+      </c>
+      <c r="C467" t="n">
+        <v>101.4</v>
+      </c>
+      <c r="D467" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="E467" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F467" t="n">
+        <v>2496</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-01-28 12:15:48</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>NIFTY2620325600CE</t>
+        </is>
+      </c>
+      <c r="C468" t="n">
+        <v>110.75</v>
+      </c>
+      <c r="D468" t="n">
+        <v>111</v>
+      </c>
+      <c r="E468" t="n">
+        <v>1040</v>
+      </c>
+      <c r="F468" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>2026-01-28 12:23:07</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>NIFTY2620325100PE</t>
+        </is>
+      </c>
+      <c r="C469" t="n">
+        <v>126.25</v>
+      </c>
+      <c r="D469" t="n">
+        <v>129</v>
+      </c>
+      <c r="E469" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F469" t="n">
+        <v>4468.75</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-01-28 12:24:47</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>NIFTY2620325100PE</t>
+        </is>
+      </c>
+      <c r="C470" t="n">
+        <v>130.15</v>
+      </c>
+      <c r="D470" t="n">
+        <v>131.9</v>
+      </c>
+      <c r="E470" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F470" t="n">
+        <v>2843.75</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-01-28 12:30:10</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>NIFTY2620325050PE</t>
+        </is>
+      </c>
+      <c r="C471" t="n">
+        <v>120.9</v>
+      </c>
+      <c r="D471" t="n">
+        <v>120.55</v>
+      </c>
+      <c r="E471" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F471" t="n">
+        <v>-568.75</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-01-28 12:38:29</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>NIFTY2620325100PE</t>
+        </is>
+      </c>
+      <c r="C472" t="n">
+        <v>132.5</v>
+      </c>
+      <c r="D472" t="n">
+        <v>132.75</v>
+      </c>
+      <c r="E472" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F472" t="n">
+        <v>406.25</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-01-28 12:40:09</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>NIFTY2620325100PE</t>
+        </is>
+      </c>
+      <c r="C473" t="n">
+        <v>133.9</v>
+      </c>
+      <c r="D473" t="n">
+        <v>134</v>
+      </c>
+      <c r="E473" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F473" t="n">
+        <v>162.5</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-01-28 12:45:17</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>NIFTY2620325500CE</t>
+        </is>
+      </c>
+      <c r="C474" t="n">
+        <v>128.05</v>
+      </c>
+      <c r="D474" t="n">
+        <v>129.1</v>
+      </c>
+      <c r="E474" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F474" t="n">
+        <v>1706.25</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-01-28 12:50:38</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>NIFTY2620325050PE</t>
+        </is>
+      </c>
+      <c r="C475" t="n">
+        <v>121.7</v>
+      </c>
+      <c r="D475" t="n">
+        <v>122.9</v>
+      </c>
+      <c r="E475" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F475" t="n">
+        <v>1950</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-01-28 12:52:25</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>NIFTY2620325500CE</t>
+        </is>
+      </c>
+      <c r="C476" t="n">
+        <v>125.15</v>
+      </c>
+      <c r="D476" t="n">
+        <v>125.35</v>
+      </c>
+      <c r="E476" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F476" t="n">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-01-28 13:00:40</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>NIFTY2620325500CE</t>
+        </is>
+      </c>
+      <c r="C477" t="n">
+        <v>126.2</v>
+      </c>
+      <c r="D477" t="n">
+        <v>119.75</v>
+      </c>
+      <c r="E477" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F477" t="n">
+        <v>-10481.25</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-01-28 13:06:38</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>NIFTY2620325100PE</t>
+        </is>
+      </c>
+      <c r="C478" t="n">
+        <v>136</v>
+      </c>
+      <c r="D478" t="n">
+        <v>137.05</v>
+      </c>
+      <c r="E478" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F478" t="n">
+        <v>1706.25</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>2026-01-28 13:08:46</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>NIFTY2620325050PE</t>
+        </is>
+      </c>
+      <c r="C479" t="n">
+        <v>120.5</v>
+      </c>
+      <c r="D479" t="n">
+        <v>120.75</v>
+      </c>
+      <c r="E479" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F479" t="n">
+        <v>406.25</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-01-28 13:27:21</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>NIFTY2620325450CE</t>
+        </is>
+      </c>
+      <c r="C480" t="n">
+        <v>132.25</v>
+      </c>
+      <c r="D480" t="n">
+        <v>132.2</v>
+      </c>
+      <c r="E480" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F480" t="n">
+        <v>-81.25</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-01-28 13:40:35</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>NIFTY2620325450CE</t>
+        </is>
+      </c>
+      <c r="C481" t="n">
+        <v>131.35</v>
+      </c>
+      <c r="D481" t="n">
+        <v>132.3</v>
+      </c>
+      <c r="E481" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F481" t="n">
+        <v>1543.75</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-01-28 13:42:10</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>NIFTY2620325050PE</t>
+        </is>
+      </c>
+      <c r="C482" t="n">
+        <v>130.45</v>
+      </c>
+      <c r="D482" t="n">
+        <v>131.45</v>
+      </c>
+      <c r="E482" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F482" t="n">
+        <v>1625</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-01-28 13:48:02</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>NIFTY2620324950PE</t>
+        </is>
+      </c>
+      <c r="C483" t="n">
+        <v>112.2</v>
+      </c>
+      <c r="D483" t="n">
+        <v>112.4</v>
+      </c>
+      <c r="E483" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F483" t="n">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-01-28 13:53:54</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>NIFTY2620325450CE</t>
+        </is>
+      </c>
+      <c r="C484" t="n">
+        <v>122.05</v>
+      </c>
+      <c r="D484" t="n">
+        <v>123.3</v>
+      </c>
+      <c r="E484" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F484" t="n">
+        <v>2031.25</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-01-28 13:55:42</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>NIFTY2620325450CE</t>
+        </is>
+      </c>
+      <c r="C485" t="n">
+        <v>125.1</v>
+      </c>
+      <c r="D485" t="n">
+        <v>125.45</v>
+      </c>
+      <c r="E485" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F485" t="n">
+        <v>568.75</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-01-28 13:58:33</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>NIFTY2620325000PE</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>121.6</v>
+      </c>
+      <c r="D486" t="n">
+        <v>115.5</v>
+      </c>
+      <c r="E486" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F486" t="n">
+        <v>-9912.5</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-01-28 14:03:27</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>NIFTY2620325050PE</t>
+        </is>
+      </c>
+      <c r="C487" t="n">
+        <v>131.8</v>
+      </c>
+      <c r="D487" t="n">
+        <v>125.7</v>
+      </c>
+      <c r="E487" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F487" t="n">
+        <v>-9912.5</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-01-28 14:05:44</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>NIFTY2620324950PE</t>
+        </is>
+      </c>
+      <c r="C488" t="n">
+        <v>99.75</v>
+      </c>
+      <c r="D488" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="E488" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F488" t="n">
+        <v>3168.75</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-01-28 14:11:43</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>NIFTY2620325050PE</t>
+        </is>
+      </c>
+      <c r="C489" t="n">
+        <v>131.5</v>
+      </c>
+      <c r="D489" t="n">
+        <v>131.75</v>
+      </c>
+      <c r="E489" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F489" t="n">
+        <v>406.25</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-01-28 14:13:18</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>NIFTY2620325000PE</t>
+        </is>
+      </c>
+      <c r="C490" t="n">
+        <v>122</v>
+      </c>
+      <c r="D490" t="n">
+        <v>122</v>
+      </c>
+      <c r="E490" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F490" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-01-28 14:14:56</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>NIFTY2620325050PE</t>
+        </is>
+      </c>
+      <c r="C491" t="n">
+        <v>134.9</v>
+      </c>
+      <c r="D491" t="n">
+        <v>135.25</v>
+      </c>
+      <c r="E491" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F491" t="n">
+        <v>568.75</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-01-28 14:18:49</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>NIFTY2620325000PE</t>
+        </is>
+      </c>
+      <c r="C492" t="n">
+        <v>123.3</v>
+      </c>
+      <c r="D492" t="n">
+        <v>123.1</v>
+      </c>
+      <c r="E492" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F492" t="n">
+        <v>-325</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-01-28 14:27:51</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>NIFTY2620325450CE</t>
+        </is>
+      </c>
+      <c r="C493" t="n">
+        <v>124.25</v>
+      </c>
+      <c r="D493" t="n">
+        <v>124.7</v>
+      </c>
+      <c r="E493" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F493" t="n">
+        <v>731.25</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-01-28 14:29:50</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>NIFTY2620325450CE</t>
+        </is>
+      </c>
+      <c r="C494" t="n">
+        <v>126.95</v>
+      </c>
+      <c r="D494" t="n">
+        <v>128.75</v>
+      </c>
+      <c r="E494" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F494" t="n">
+        <v>2925</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-01-28 14:31:38</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>NIFTY2620325450CE</t>
+        </is>
+      </c>
+      <c r="C495" t="n">
+        <v>133.4</v>
+      </c>
+      <c r="D495" t="n">
+        <v>133.65</v>
+      </c>
+      <c r="E495" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F495" t="n">
+        <v>406.25</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-01-28 14:36:40</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>NIFTY2620325050PE</t>
+        </is>
+      </c>
+      <c r="C496" t="n">
+        <v>130</v>
+      </c>
+      <c r="D496" t="n">
+        <v>132</v>
+      </c>
+      <c r="E496" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F496" t="n">
+        <v>3250</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-01-28 14:43:18</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>NIFTY2620325050PE</t>
+        </is>
+      </c>
+      <c r="C497" t="n">
+        <v>127.35</v>
+      </c>
+      <c r="D497" t="n">
+        <v>121.2</v>
+      </c>
+      <c r="E497" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F497" t="n">
+        <v>-9993.75</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-01-28 14:44:15</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>NIFTY2620325550CE</t>
+        </is>
+      </c>
+      <c r="C498" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="D498" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="E498" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F498" t="n">
+        <v>893.75</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>2026-01-28 14:54:11</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>NIFTY2620325500CE</t>
+        </is>
+      </c>
+      <c r="C499" t="n">
+        <v>134.9</v>
+      </c>
+      <c r="D499" t="n">
+        <v>138.85</v>
+      </c>
+      <c r="E499" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F499" t="n">
+        <v>6418.75</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-01-29 11:55:12</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>NIFTY2620325100PE</t>
+        </is>
+      </c>
+      <c r="C500" t="n">
+        <v>123.85</v>
+      </c>
+      <c r="D500" t="n">
+        <v>123.15</v>
+      </c>
+      <c r="E500" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F500" t="n">
+        <v>-1137.5</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-01-29 12:05:40</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>NIFTY2620325150PE</t>
+        </is>
+      </c>
+      <c r="C501" t="n">
+        <v>136.1</v>
+      </c>
+      <c r="D501" t="n">
+        <v>130.1</v>
+      </c>
+      <c r="E501" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F501" t="n">
+        <v>-9750</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-01-29 12:10:19</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>NIFTY2620325450CE</t>
+        </is>
+      </c>
+      <c r="C502" t="n">
+        <v>124.55</v>
+      </c>
+      <c r="D502" t="n">
+        <v>124.4</v>
+      </c>
+      <c r="E502" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F502" t="n">
+        <v>-243.75</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-01-29 12:17:30</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>NIFTY2620325450CE</t>
+        </is>
+      </c>
+      <c r="C503" t="n">
+        <v>123.25</v>
+      </c>
+      <c r="D503" t="n">
+        <v>117.15</v>
+      </c>
+      <c r="E503" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F503" t="n">
+        <v>-9912.5</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-01-30 10:42:46</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>NIFTY2620325450CE</t>
+        </is>
+      </c>
+      <c r="C504" t="n">
+        <v>137.4</v>
+      </c>
+      <c r="D504" t="n">
+        <v>135.25</v>
+      </c>
+      <c r="E504" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F504" t="n">
+        <v>-3493.75</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-01-30 10:58:44</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>NIFTY2620325450CE</t>
+        </is>
+      </c>
+      <c r="C505" t="n">
+        <v>134.55</v>
+      </c>
+      <c r="D505" t="n">
+        <v>135.6</v>
+      </c>
+      <c r="E505" t="n">
+        <v>1625</v>
+      </c>
+      <c r="F505" t="n">
+        <v>1706.25</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:40:49</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C506" t="n">
+        <v>107.05</v>
+      </c>
+      <c r="D506" t="n">
+        <v>107.65</v>
+      </c>
+      <c r="E506" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F506" t="n">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:40:50</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C507" t="n">
+        <v>107.05</v>
+      </c>
+      <c r="D507" t="n">
+        <v>107.65</v>
+      </c>
+      <c r="E507" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F507" t="n">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:40:52</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C508" t="n">
+        <v>107.05</v>
+      </c>
+      <c r="D508" t="n">
+        <v>107.85</v>
+      </c>
+      <c r="E508" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F508" t="n">
+        <v>1144</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:40:57</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C509" t="n">
+        <v>107.05</v>
+      </c>
+      <c r="D509" t="n">
+        <v>108.25</v>
+      </c>
+      <c r="E509" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F509" t="n">
+        <v>1716</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:41:00</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C510" t="n">
+        <v>107.05</v>
+      </c>
+      <c r="D510" t="n">
+        <v>108.25</v>
+      </c>
+      <c r="E510" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F510" t="n">
+        <v>1716</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:42:18</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C511" t="n">
+        <v>107.05</v>
+      </c>
+      <c r="D511" t="n">
+        <v>104.7</v>
+      </c>
+      <c r="E511" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F511" t="n">
+        <v>-3360.5</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:43:35</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C512" t="n">
+        <v>107.05</v>
+      </c>
+      <c r="D512" t="n">
+        <v>102.05</v>
+      </c>
+      <c r="E512" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F512" t="n">
+        <v>-7150</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:43:37</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C513" t="n">
+        <v>107.05</v>
+      </c>
+      <c r="D513" t="n">
+        <v>105.35</v>
+      </c>
+      <c r="E513" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F513" t="n">
+        <v>-2431</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:43:39</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C514" t="n">
+        <v>107.05</v>
+      </c>
+      <c r="D514" t="n">
+        <v>104.6</v>
+      </c>
+      <c r="E514" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F514" t="n">
+        <v>-3503.5</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:26</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C515" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D515" t="n">
+        <v>102.3</v>
+      </c>
+      <c r="E515" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F515" t="n">
+        <v>1215.5</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:26</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C516" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D516" t="n">
+        <v>101.75</v>
+      </c>
+      <c r="E516" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F516" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:27</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C517" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D517" t="n">
+        <v>101.1</v>
+      </c>
+      <c r="E517" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F517" t="n">
+        <v>-500.5</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:27</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C518" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D518" t="n">
+        <v>101.75</v>
+      </c>
+      <c r="E518" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F518" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:27</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C519" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D519" t="n">
+        <v>102.25</v>
+      </c>
+      <c r="E519" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F519" t="n">
+        <v>1144</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:28</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C520" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D520" t="n">
+        <v>101.75</v>
+      </c>
+      <c r="E520" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F520" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:30</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C521" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D521" t="n">
+        <v>103.1</v>
+      </c>
+      <c r="E521" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F521" t="n">
+        <v>2359.5</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:32</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C522" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D522" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="E522" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F522" t="n">
+        <v>1930.5</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:34</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C523" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D523" t="n">
+        <v>103</v>
+      </c>
+      <c r="E523" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F523" t="n">
+        <v>2216.5</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:35</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C524" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D524" t="n">
+        <v>101.65</v>
+      </c>
+      <c r="E524" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F524" t="n">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:38</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C525" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D525" t="n">
+        <v>101.55</v>
+      </c>
+      <c r="E525" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F525" t="n">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:40</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C526" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D526" t="n">
+        <v>101.55</v>
+      </c>
+      <c r="E526" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F526" t="n">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:42</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C527" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D527" t="n">
+        <v>99.84999999999999</v>
+      </c>
+      <c r="E527" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F527" t="n">
+        <v>-2288</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:43</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C528" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D528" t="n">
+        <v>98.55</v>
+      </c>
+      <c r="E528" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F528" t="n">
+        <v>-4147</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:44</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C529" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D529" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="E529" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F529" t="n">
+        <v>-3789.5</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:46</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C530" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D530" t="n">
+        <v>98.8</v>
+      </c>
+      <c r="E530" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F530" t="n">
+        <v>-3789.5</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:47</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C531" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D531" t="n">
+        <v>97.95</v>
+      </c>
+      <c r="E531" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F531" t="n">
+        <v>-5005</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:48</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C532" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D532" t="n">
+        <v>97.55</v>
+      </c>
+      <c r="E532" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F532" t="n">
+        <v>-5577</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:50</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C533" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D533" t="n">
+        <v>97.45</v>
+      </c>
+      <c r="E533" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F533" t="n">
+        <v>-5720</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:51</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C534" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D534" t="n">
+        <v>97.45</v>
+      </c>
+      <c r="E534" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F534" t="n">
+        <v>-5720</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:53</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C535" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D535" t="n">
+        <v>98.15000000000001</v>
+      </c>
+      <c r="E535" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F535" t="n">
+        <v>-4719</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:46:54</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C536" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D536" t="n">
+        <v>99.2</v>
+      </c>
+      <c r="E536" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F536" t="n">
+        <v>-3217.5</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:48:11</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C537" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="D537" t="n">
+        <v>99.2</v>
+      </c>
+      <c r="E537" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F537" t="n">
+        <v>-3217.5</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026-02-02 12:54:06</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C538" t="n">
+        <v>112.75</v>
+      </c>
+      <c r="D538" t="n">
+        <v>112.7</v>
+      </c>
+      <c r="E538" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F538" t="n">
+        <v>-71.5</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:06:32</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C539" t="n">
+        <v>140.7</v>
+      </c>
+      <c r="D539" t="n">
+        <v>152.5</v>
+      </c>
+      <c r="E539" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F539" t="n">
+        <v>16874</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:08:21</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C540" t="n">
+        <v>151.05</v>
+      </c>
+      <c r="D540" t="n">
+        <v>151.55</v>
+      </c>
+      <c r="E540" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F540" t="n">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:10:35</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C541" t="n">
+        <v>151.4</v>
+      </c>
+      <c r="D541" t="n">
+        <v>150.9</v>
+      </c>
+      <c r="E541" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F541" t="n">
+        <v>-715</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:13:38</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900PE</t>
+        </is>
+      </c>
+      <c r="C542" t="n">
+        <v>95.95</v>
+      </c>
+      <c r="D542" t="n">
+        <v>98.09999999999999</v>
+      </c>
+      <c r="E542" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F542" t="n">
+        <v>3074.5</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:14:14</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900CE</t>
+        </is>
+      </c>
+      <c r="C543" t="n">
+        <v>132.6</v>
+      </c>
+      <c r="D543" t="n">
+        <v>137.35</v>
+      </c>
+      <c r="E543" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F543" t="n">
+        <v>6792.5</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:16:14</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900PE</t>
+        </is>
+      </c>
+      <c r="C544" t="n">
+        <v>98.75</v>
+      </c>
+      <c r="D544" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="E544" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F544" t="n">
+        <v>929.5</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:16:48</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900PE</t>
+        </is>
+      </c>
+      <c r="C545" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="D545" t="n">
+        <v>108</v>
+      </c>
+      <c r="E545" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F545" t="n">
+        <v>6721</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:17:25</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900PE</t>
+        </is>
+      </c>
+      <c r="C546" t="n">
+        <v>103.85</v>
+      </c>
+      <c r="D546" t="n">
+        <v>104.1</v>
+      </c>
+      <c r="E546" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F546" t="n">
+        <v>357.5</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:19:03</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900PE</t>
+        </is>
+      </c>
+      <c r="C547" t="n">
+        <v>113.25</v>
+      </c>
+      <c r="D547" t="n">
+        <v>114.3</v>
+      </c>
+      <c r="E547" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F547" t="n">
+        <v>1501.5</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:19:30</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900PE</t>
+        </is>
+      </c>
+      <c r="C548" t="n">
+        <v>118.35</v>
+      </c>
+      <c r="D548" t="n">
+        <v>119.15</v>
+      </c>
+      <c r="E548" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F548" t="n">
+        <v>1144</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:20:39</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900PE</t>
+        </is>
+      </c>
+      <c r="C549" t="n">
+        <v>122.6</v>
+      </c>
+      <c r="D549" t="n">
+        <v>123.5</v>
+      </c>
+      <c r="E549" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F549" t="n">
+        <v>1287</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:22:09</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900PE</t>
+        </is>
+      </c>
+      <c r="C550" t="n">
+        <v>125.75</v>
+      </c>
+      <c r="D550" t="n">
+        <v>128.05</v>
+      </c>
+      <c r="E550" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F550" t="n">
+        <v>3289</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-02-02 13:25:32</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>NIFTY2620324900PE</t>
+        </is>
+      </c>
+      <c r="C551" t="n">
+        <v>127.75</v>
+      </c>
+      <c r="D551" t="n">
+        <v>133.7</v>
+      </c>
+      <c r="E551" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F551" t="n">
+        <v>8508.5</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-02-05 12:52:55</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>NIFTY2621025700CE</t>
+        </is>
+      </c>
+      <c r="C552" t="n">
+        <v>116.3</v>
+      </c>
+      <c r="D552" t="n">
+        <v>116.4</v>
+      </c>
+      <c r="E552" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F552" t="n">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026-02-06 10:31:41</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>NIFTY2621025500PE</t>
+        </is>
+      </c>
+      <c r="C553" t="n">
+        <v>104.35</v>
+      </c>
+      <c r="D553" t="n">
+        <v>106.8</v>
+      </c>
+      <c r="E553" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F553" t="n">
+        <v>3503.5</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-02-06 10:32:25</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>NIFTY2621025500PE</t>
+        </is>
+      </c>
+      <c r="C554" t="n">
+        <v>103.1</v>
+      </c>
+      <c r="D554" t="n">
+        <v>103.55</v>
+      </c>
+      <c r="E554" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F554" t="n">
+        <v>643.5</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026-02-06 10:37:13</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>NIFTY2621025500CE</t>
+        </is>
+      </c>
+      <c r="C555" t="n">
+        <v>124.5</v>
+      </c>
+      <c r="D555" t="n">
+        <v>127.35</v>
+      </c>
+      <c r="E555" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F555" t="n">
+        <v>4075.5</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026-02-06 10:40:02</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>NIFTY2621025500CE</t>
+        </is>
+      </c>
+      <c r="C556" t="n">
+        <v>126.8</v>
+      </c>
+      <c r="D556" t="n">
+        <v>127.65</v>
+      </c>
+      <c r="E556" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F556" t="n">
+        <v>1215.5</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026-02-06 10:41:27</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>NIFTY2621025500PE</t>
+        </is>
+      </c>
+      <c r="C557" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="D557" t="n">
+        <v>105.15</v>
+      </c>
+      <c r="E557" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F557" t="n">
+        <v>2788.5</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026-02-06 10:44:00</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>NIFTY2621025500PE</t>
+        </is>
+      </c>
+      <c r="C558" t="n">
+        <v>108.1</v>
+      </c>
+      <c r="D558" t="n">
+        <v>108.2</v>
+      </c>
+      <c r="E558" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F558" t="n">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026-02-06 10:44:58</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>NIFTY2621025500PE</t>
+        </is>
+      </c>
+      <c r="C559" t="n">
+        <v>108.05</v>
+      </c>
+      <c r="D559" t="n">
+        <v>108.4</v>
+      </c>
+      <c r="E559" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F559" t="n">
+        <v>500.5</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026-02-06 11:25:04</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>NIFTY2621025500CE</t>
+        </is>
+      </c>
+      <c r="C560" t="n">
+        <v>162.7</v>
+      </c>
+      <c r="D560" t="n">
+        <v>164.4</v>
+      </c>
+      <c r="E560" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F560" t="n">
+        <v>2431</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-02-06 11:26:09</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>NIFTY2621025600CE</t>
+        </is>
+      </c>
+      <c r="C561" t="n">
+        <v>108.4</v>
+      </c>
+      <c r="D561" t="n">
+        <v>107.85</v>
+      </c>
+      <c r="E561" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F561" t="n">
+        <v>-786.5</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026-02-06 11:26:37</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>NIFTY2621025600CE</t>
+        </is>
+      </c>
+      <c r="C562" t="n">
+        <v>107.35</v>
+      </c>
+      <c r="D562" t="n">
+        <v>106.6</v>
+      </c>
+      <c r="E562" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F562" t="n">
+        <v>-1072.5</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026-02-06 11:27:19</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>NIFTY2621025600CE</t>
+        </is>
+      </c>
+      <c r="C563" t="n">
+        <v>108.2</v>
+      </c>
+      <c r="D563" t="n">
+        <v>108.45</v>
+      </c>
+      <c r="E563" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F563" t="n">
+        <v>357.5</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026-02-06 11:27:51</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>NIFTY2621025600PE</t>
+        </is>
+      </c>
+      <c r="C564" t="n">
+        <v>114.15</v>
+      </c>
+      <c r="D564" t="n">
+        <v>113.15</v>
+      </c>
+      <c r="E564" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F564" t="n">
+        <v>-1430</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
introduces new manual bot name PROD10-,very efficient for intraday
</commit_message>
<xml_diff>
--- a/Lakshmi.xlsx
+++ b/Lakshmi.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H564"/>
+  <dimension ref="A1:H658"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="24.33203125" customWidth="1" style="1" min="1" max="1"/>
@@ -16725,6 +16725,2262 @@
       </c>
       <c r="F564" t="n">
         <v>-1430</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026-02-09 11:22:44</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>NIFTY2621025800CE</t>
+        </is>
+      </c>
+      <c r="C565" t="n">
+        <v>119</v>
+      </c>
+      <c r="D565" t="n">
+        <v>120.9</v>
+      </c>
+      <c r="E565" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F565" t="n">
+        <v>2717</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026-02-09 11:25:24</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>NIFTY2621025800CE</t>
+        </is>
+      </c>
+      <c r="C566" t="n">
+        <v>122.85</v>
+      </c>
+      <c r="D566" t="n">
+        <v>124.4</v>
+      </c>
+      <c r="E566" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F566" t="n">
+        <v>2216.5</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026-02-11 12:30:17</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>SENSEX2621283500CE</t>
+        </is>
+      </c>
+      <c r="C567" t="n">
+        <v>795.9</v>
+      </c>
+      <c r="D567" t="n">
+        <v>794</v>
+      </c>
+      <c r="E567" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F567" t="n">
+        <v>-1900</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026-02-11 12:31:39</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>SENSEX2621284500CE</t>
+        </is>
+      </c>
+      <c r="C568" t="n">
+        <v>104.7</v>
+      </c>
+      <c r="D568" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="E568" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F568" t="n">
+        <v>-1200</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026-02-11 12:32:51</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>SENSEX2621284000PE</t>
+        </is>
+      </c>
+      <c r="C569" t="n">
+        <v>105.9</v>
+      </c>
+      <c r="D569" t="n">
+        <v>113.35</v>
+      </c>
+      <c r="E569" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F569" t="n">
+        <v>7450</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026-02-11 12:37:57</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>SENSEX2621283900PE</t>
+        </is>
+      </c>
+      <c r="C570" t="n">
+        <v>91.15000000000001</v>
+      </c>
+      <c r="D570" t="n">
+        <v>99</v>
+      </c>
+      <c r="E570" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F570" t="n">
+        <v>7850</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026-02-11 12:38:44</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>SENSEX2621283900PE</t>
+        </is>
+      </c>
+      <c r="C571" t="n">
+        <v>97.25</v>
+      </c>
+      <c r="D571" t="n">
+        <v>96.15000000000001</v>
+      </c>
+      <c r="E571" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F571" t="n">
+        <v>-1100</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026-02-11 12:40:28</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>SENSEX2621283900PE</t>
+        </is>
+      </c>
+      <c r="C572" t="n">
+        <v>101</v>
+      </c>
+      <c r="D572" t="n">
+        <v>99.7</v>
+      </c>
+      <c r="E572" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F572" t="n">
+        <v>-1300</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026-02-12 11:43:01</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>SENSEX2621283800CE</t>
+        </is>
+      </c>
+      <c r="C573" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="D573" t="n">
+        <v>101.3</v>
+      </c>
+      <c r="E573" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F573" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026-02-12 11:46:18</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>SENSEX2621283800CE</t>
+        </is>
+      </c>
+      <c r="C574" t="n">
+        <v>99.95</v>
+      </c>
+      <c r="D574" t="n">
+        <v>100.3</v>
+      </c>
+      <c r="E574" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F574" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>2026-02-12 11:46:40</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>SENSEX2621283800CE</t>
+        </is>
+      </c>
+      <c r="C575" t="n">
+        <v>100.35</v>
+      </c>
+      <c r="D575" t="n">
+        <v>99.7</v>
+      </c>
+      <c r="E575" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F575" t="n">
+        <v>-650</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026-02-13 11:34:01</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>NIFTY2621725550PE</t>
+        </is>
+      </c>
+      <c r="C576" t="n">
+        <v>93.59999999999999</v>
+      </c>
+      <c r="D576" t="n">
+        <v>95.45</v>
+      </c>
+      <c r="E576" t="n">
+        <v>975</v>
+      </c>
+      <c r="F576" t="n">
+        <v>1803.75</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026-02-13 11:35:12</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>NIFTY2621725550PE</t>
+        </is>
+      </c>
+      <c r="C577" t="n">
+        <v>96.75</v>
+      </c>
+      <c r="D577" t="n">
+        <v>98.25</v>
+      </c>
+      <c r="E577" t="n">
+        <v>975</v>
+      </c>
+      <c r="F577" t="n">
+        <v>1462.5</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026-02-16 12:18:30</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>NIFTY2621725550CE</t>
+        </is>
+      </c>
+      <c r="C578" t="n">
+        <v>87.65000000000001</v>
+      </c>
+      <c r="D578" t="n">
+        <v>87.3</v>
+      </c>
+      <c r="E578" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F578" t="n">
+        <v>-500.5</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>2026-02-16 12:19:15</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>NIFTY2621725500CE</t>
+        </is>
+      </c>
+      <c r="C579" t="n">
+        <v>122</v>
+      </c>
+      <c r="D579" t="n">
+        <v>122.4</v>
+      </c>
+      <c r="E579" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F579" t="n">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026-02-16 12:20:15</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>NIFTY2621725500CE</t>
+        </is>
+      </c>
+      <c r="C580" t="n">
+        <v>122.15</v>
+      </c>
+      <c r="D580" t="n">
+        <v>122.6</v>
+      </c>
+      <c r="E580" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F580" t="n">
+        <v>643.5</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026-02-16 12:35:57</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>NIFTY2621725500CE</t>
+        </is>
+      </c>
+      <c r="C581" t="n">
+        <v>133.45</v>
+      </c>
+      <c r="D581" t="n">
+        <v>135.45</v>
+      </c>
+      <c r="E581" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F581" t="n">
+        <v>2860</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026-02-16 12:50:01</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>NIFTY2621725650PE</t>
+        </is>
+      </c>
+      <c r="C582" t="n">
+        <v>118.75</v>
+      </c>
+      <c r="D582" t="n">
+        <v>125.05</v>
+      </c>
+      <c r="E582" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F582" t="n">
+        <v>9009</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026-02-16 12:53:38</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>NIFTY2621725500CE</t>
+        </is>
+      </c>
+      <c r="C583" t="n">
+        <v>122.7</v>
+      </c>
+      <c r="D583" t="n">
+        <v>125.7</v>
+      </c>
+      <c r="E583" t="n">
+        <v>1430</v>
+      </c>
+      <c r="F583" t="n">
+        <v>4290</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026-02-17 09:50:57</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25750CE</t>
+        </is>
+      </c>
+      <c r="C584" t="n">
+        <v>118.75</v>
+      </c>
+      <c r="D584" t="n">
+        <v>118.6</v>
+      </c>
+      <c r="E584" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F584" t="n">
+        <v>-195</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026-02-17 09:52:40</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>NIFTY2621725550CE</t>
+        </is>
+      </c>
+      <c r="C585" t="n">
+        <v>117.15</v>
+      </c>
+      <c r="D585" t="n">
+        <v>123.2</v>
+      </c>
+      <c r="E585" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F585" t="n">
+        <v>7865</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026-02-17 09:53:27</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25750CE</t>
+        </is>
+      </c>
+      <c r="C586" t="n">
+        <v>123.9</v>
+      </c>
+      <c r="D586" t="n">
+        <v>124.65</v>
+      </c>
+      <c r="E586" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F586" t="n">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026-02-17 09:54:06</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25750CE</t>
+        </is>
+      </c>
+      <c r="C587" t="n">
+        <v>123.8</v>
+      </c>
+      <c r="D587" t="n">
+        <v>124</v>
+      </c>
+      <c r="E587" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F587" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026-02-17 09:57:39</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25750CE</t>
+        </is>
+      </c>
+      <c r="C588" t="n">
+        <v>124.75</v>
+      </c>
+      <c r="D588" t="n">
+        <v>125.25</v>
+      </c>
+      <c r="E588" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F588" t="n">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2026-02-17 10:09:12</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25750CE</t>
+        </is>
+      </c>
+      <c r="C589" t="n">
+        <v>128.6</v>
+      </c>
+      <c r="D589" t="n">
+        <v>129.45</v>
+      </c>
+      <c r="E589" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F589" t="n">
+        <v>1105</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026-02-17 10:26:39</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25750CE</t>
+        </is>
+      </c>
+      <c r="C590" t="n">
+        <v>139.8</v>
+      </c>
+      <c r="D590" t="n">
+        <v>139.8</v>
+      </c>
+      <c r="E590" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F590" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026-02-17 10:27:03</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25750CE</t>
+        </is>
+      </c>
+      <c r="C591" t="n">
+        <v>148.65</v>
+      </c>
+      <c r="D591" t="n">
+        <v>148.75</v>
+      </c>
+      <c r="E591" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F591" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026-02-17 10:27:26</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25750CE</t>
+        </is>
+      </c>
+      <c r="C592" t="n">
+        <v>151</v>
+      </c>
+      <c r="D592" t="n">
+        <v>151</v>
+      </c>
+      <c r="E592" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F592" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026-02-17 10:27:59</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25750CE</t>
+        </is>
+      </c>
+      <c r="C593" t="n">
+        <v>154.7</v>
+      </c>
+      <c r="D593" t="n">
+        <v>155.35</v>
+      </c>
+      <c r="E593" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F593" t="n">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026-02-17 10:29:05</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>NIFTY2621725650CE</t>
+        </is>
+      </c>
+      <c r="C594" t="n">
+        <v>98</v>
+      </c>
+      <c r="D594" t="n">
+        <v>103.05</v>
+      </c>
+      <c r="E594" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F594" t="n">
+        <v>6565</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026-02-17 10:32:41</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>NIFTY2621725650CE</t>
+        </is>
+      </c>
+      <c r="C595" t="n">
+        <v>101.85</v>
+      </c>
+      <c r="D595" t="n">
+        <v>102.45</v>
+      </c>
+      <c r="E595" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F595" t="n">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026-02-17 10:36:05</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>NIFTY2621725800PE</t>
+        </is>
+      </c>
+      <c r="C596" t="n">
+        <v>111.95</v>
+      </c>
+      <c r="D596" t="n">
+        <v>111.8</v>
+      </c>
+      <c r="E596" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F596" t="n">
+        <v>-195</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026-02-17 10:36:29</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>NIFTY2621725800PE</t>
+        </is>
+      </c>
+      <c r="C597" t="n">
+        <v>110.65</v>
+      </c>
+      <c r="D597" t="n">
+        <v>110.6</v>
+      </c>
+      <c r="E597" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F597" t="n">
+        <v>-65</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026-02-17 10:37:28</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>NIFTY2621725800PE</t>
+        </is>
+      </c>
+      <c r="C598" t="n">
+        <v>113.25</v>
+      </c>
+      <c r="D598" t="n">
+        <v>112.2</v>
+      </c>
+      <c r="E598" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F598" t="n">
+        <v>-1365</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>2026-02-17 10:38:01</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>NIFTY2621725800PE</t>
+        </is>
+      </c>
+      <c r="C599" t="n">
+        <v>114.9</v>
+      </c>
+      <c r="D599" t="n">
+        <v>117.35</v>
+      </c>
+      <c r="E599" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F599" t="n">
+        <v>3185</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026-02-17 10:40:45</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>NIFTY2621725800PE</t>
+        </is>
+      </c>
+      <c r="C600" t="n">
+        <v>120.5</v>
+      </c>
+      <c r="D600" t="n">
+        <v>122.35</v>
+      </c>
+      <c r="E600" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F600" t="n">
+        <v>2405</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026-02-17 10:41:51</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>NIFTY2621725800PE</t>
+        </is>
+      </c>
+      <c r="C601" t="n">
+        <v>121.6</v>
+      </c>
+      <c r="D601" t="n">
+        <v>122.6</v>
+      </c>
+      <c r="E601" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F601" t="n">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>2026-02-17 10:43:38</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>NIFTY2621725800PE</t>
+        </is>
+      </c>
+      <c r="C602" t="n">
+        <v>127.85</v>
+      </c>
+      <c r="D602" t="n">
+        <v>134.25</v>
+      </c>
+      <c r="E602" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F602" t="n">
+        <v>8320</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>2026-02-17 11:33:11</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>NIFTY2621725600CE</t>
+        </is>
+      </c>
+      <c r="C603" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="D603" t="n">
+        <v>114.45</v>
+      </c>
+      <c r="E603" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F603" t="n">
+        <v>15535</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>2026-02-17 12:40:30</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>NIFTY2621725850PE</t>
+        </is>
+      </c>
+      <c r="C604" t="n">
+        <v>125.1</v>
+      </c>
+      <c r="D604" t="n">
+        <v>116.2</v>
+      </c>
+      <c r="E604" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F604" t="n">
+        <v>-11570</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>2026-02-18 09:47:31</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25700PE</t>
+        </is>
+      </c>
+      <c r="C605" t="n">
+        <v>115.3</v>
+      </c>
+      <c r="D605" t="n">
+        <v>116.15</v>
+      </c>
+      <c r="E605" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F605" t="n">
+        <v>1105</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>2026-02-18 09:53:15</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25700PE</t>
+        </is>
+      </c>
+      <c r="C606" t="n">
+        <v>119.75</v>
+      </c>
+      <c r="D606" t="n">
+        <v>122.85</v>
+      </c>
+      <c r="E606" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F606" t="n">
+        <v>4030</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>2026-02-18 09:54:59</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25700PE</t>
+        </is>
+      </c>
+      <c r="C607" t="n">
+        <v>127.3</v>
+      </c>
+      <c r="D607" t="n">
+        <v>127.1</v>
+      </c>
+      <c r="E607" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F607" t="n">
+        <v>-260</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>2026-02-18 09:55:30</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25700PE</t>
+        </is>
+      </c>
+      <c r="C608" t="n">
+        <v>129.8</v>
+      </c>
+      <c r="D608" t="n">
+        <v>131.5</v>
+      </c>
+      <c r="E608" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F608" t="n">
+        <v>2210</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>2026-02-18 09:56:04</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25700PE</t>
+        </is>
+      </c>
+      <c r="C609" t="n">
+        <v>135</v>
+      </c>
+      <c r="D609" t="n">
+        <v>141.75</v>
+      </c>
+      <c r="E609" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F609" t="n">
+        <v>8775</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>2026-02-18 10:18:12</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25600PE</t>
+        </is>
+      </c>
+      <c r="C610" t="n">
+        <v>115.2</v>
+      </c>
+      <c r="D610" t="n">
+        <v>108</v>
+      </c>
+      <c r="E610" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F610" t="n">
+        <v>-9360</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>2026-02-18 10:34:16</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25750CE</t>
+        </is>
+      </c>
+      <c r="C611" t="n">
+        <v>109.9</v>
+      </c>
+      <c r="D611" t="n">
+        <v>110.15</v>
+      </c>
+      <c r="E611" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F611" t="n">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>2026-02-18 10:37:11</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25600PE</t>
+        </is>
+      </c>
+      <c r="C612" t="n">
+        <v>101.35</v>
+      </c>
+      <c r="D612" t="n">
+        <v>95.3</v>
+      </c>
+      <c r="E612" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F612" t="n">
+        <v>-7865</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>2026-02-20 10:58:33</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C613" t="n">
+        <v>117.9</v>
+      </c>
+      <c r="D613" t="n">
+        <v>108.85</v>
+      </c>
+      <c r="E613" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F613" t="n">
+        <v>-11765</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>2026-02-20 10:59:33</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C614" t="n">
+        <v>109.7</v>
+      </c>
+      <c r="D614" t="n">
+        <v>113.1</v>
+      </c>
+      <c r="E614" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F614" t="n">
+        <v>4420</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>2026-02-20 11:01:04</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C615" t="n">
+        <v>114.85</v>
+      </c>
+      <c r="D615" t="n">
+        <v>115.7</v>
+      </c>
+      <c r="E615" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F615" t="n">
+        <v>1105</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>2026-02-20 11:07:42</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C616" t="n">
+        <v>109.85</v>
+      </c>
+      <c r="D616" t="n">
+        <v>111.85</v>
+      </c>
+      <c r="E616" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F616" t="n">
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>2026-02-20 11:13:17</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C617" t="n">
+        <v>114.15</v>
+      </c>
+      <c r="D617" t="n">
+        <v>114.45</v>
+      </c>
+      <c r="E617" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F617" t="n">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>2026-02-20 11:14:10</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C618" t="n">
+        <v>113.65</v>
+      </c>
+      <c r="D618" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="E618" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F618" t="n">
+        <v>-12025</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>2026-02-20 11:14:49</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25550PE</t>
+        </is>
+      </c>
+      <c r="C619" t="n">
+        <v>120.4</v>
+      </c>
+      <c r="D619" t="n">
+        <v>121.15</v>
+      </c>
+      <c r="E619" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F619" t="n">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>2026-02-20 11:15:45</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C620" t="n">
+        <v>110.3</v>
+      </c>
+      <c r="D620" t="n">
+        <v>112.1</v>
+      </c>
+      <c r="E620" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F620" t="n">
+        <v>2340</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>2026-02-20 12:12:50</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C621" t="n">
+        <v>110.5</v>
+      </c>
+      <c r="D621" t="n">
+        <v>110.65</v>
+      </c>
+      <c r="E621" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F621" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>2026-02-20 12:14:22</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C622" t="n">
+        <v>112.55</v>
+      </c>
+      <c r="D622" t="n">
+        <v>114</v>
+      </c>
+      <c r="E622" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F622" t="n">
+        <v>1885</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>2026-02-20 14:35:53</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C623" t="n">
+        <v>114.65</v>
+      </c>
+      <c r="D623" t="n">
+        <v>118.6</v>
+      </c>
+      <c r="E623" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F623" t="n">
+        <v>5135</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>2026-02-20 14:36:16</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C624" t="n">
+        <v>118.95</v>
+      </c>
+      <c r="D624" t="n">
+        <v>119.1</v>
+      </c>
+      <c r="E624" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F624" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>2026-02-20 14:37:10</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C625" t="n">
+        <v>115.3</v>
+      </c>
+      <c r="D625" t="n">
+        <v>115.95</v>
+      </c>
+      <c r="E625" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F625" t="n">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>2026-02-20 14:38:26</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C626" t="n">
+        <v>111.15</v>
+      </c>
+      <c r="D626" t="n">
+        <v>112</v>
+      </c>
+      <c r="E626" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F626" t="n">
+        <v>1105</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>2026-02-20 14:39:37</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C627" t="n">
+        <v>111.85</v>
+      </c>
+      <c r="D627" t="n">
+        <v>114.1</v>
+      </c>
+      <c r="E627" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F627" t="n">
+        <v>2925</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>2026-02-20 14:40:48</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C628" t="n">
+        <v>118.45</v>
+      </c>
+      <c r="D628" t="n">
+        <v>119</v>
+      </c>
+      <c r="E628" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F628" t="n">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>2026-02-20 14:41:24</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25500CE</t>
+        </is>
+      </c>
+      <c r="C629" t="n">
+        <v>206.45</v>
+      </c>
+      <c r="D629" t="n">
+        <v>208.65</v>
+      </c>
+      <c r="E629" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F629" t="n">
+        <v>2860</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>2026-02-20 14:42:08</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25500CE</t>
+        </is>
+      </c>
+      <c r="C630" t="n">
+        <v>206.9</v>
+      </c>
+      <c r="D630" t="n">
+        <v>211</v>
+      </c>
+      <c r="E630" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F630" t="n">
+        <v>5330</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>2026-02-20 14:42:32</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25500CE</t>
+        </is>
+      </c>
+      <c r="C631" t="n">
+        <v>208.95</v>
+      </c>
+      <c r="D631" t="n">
+        <v>209.75</v>
+      </c>
+      <c r="E631" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F631" t="n">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>2026-02-20 14:43:14</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25500CE</t>
+        </is>
+      </c>
+      <c r="C632" t="n">
+        <v>209.85</v>
+      </c>
+      <c r="D632" t="n">
+        <v>212.9</v>
+      </c>
+      <c r="E632" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F632" t="n">
+        <v>3965</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>2026-02-20 14:43:36</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25500CE</t>
+        </is>
+      </c>
+      <c r="C633" t="n">
+        <v>210.9</v>
+      </c>
+      <c r="D633" t="n">
+        <v>211.4</v>
+      </c>
+      <c r="E633" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F633" t="n">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>2026-02-20 14:44:30</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25500CE</t>
+        </is>
+      </c>
+      <c r="C634" t="n">
+        <v>222.95</v>
+      </c>
+      <c r="D634" t="n">
+        <v>228.3</v>
+      </c>
+      <c r="E634" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F634" t="n">
+        <v>6955</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>2026-02-20 14:44:57</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25500CE</t>
+        </is>
+      </c>
+      <c r="C635" t="n">
+        <v>223.15</v>
+      </c>
+      <c r="D635" t="n">
+        <v>222.75</v>
+      </c>
+      <c r="E635" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F635" t="n">
+        <v>-520</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>2026-02-20 14:45:41</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25500CE</t>
+        </is>
+      </c>
+      <c r="C636" t="n">
+        <v>223.95</v>
+      </c>
+      <c r="D636" t="n">
+        <v>226.85</v>
+      </c>
+      <c r="E636" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F636" t="n">
+        <v>3770</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>2026-02-23 11:48:34</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C637" t="n">
+        <v>109.45</v>
+      </c>
+      <c r="D637" t="n">
+        <v>100.15</v>
+      </c>
+      <c r="E637" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F637" t="n">
+        <v>-12090</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>2026-02-23 11:49:42</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650PE</t>
+        </is>
+      </c>
+      <c r="C638" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="D638" t="n">
+        <v>106.75</v>
+      </c>
+      <c r="E638" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F638" t="n">
+        <v>8125</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>2026-02-23 11:50:11</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650PE</t>
+        </is>
+      </c>
+      <c r="C639" t="n">
+        <v>97</v>
+      </c>
+      <c r="D639" t="n">
+        <v>99.55</v>
+      </c>
+      <c r="E639" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F639" t="n">
+        <v>3315</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>2026-02-23 11:50:28</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650PE</t>
+        </is>
+      </c>
+      <c r="C640" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="D640" t="n">
+        <v>102.95</v>
+      </c>
+      <c r="E640" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F640" t="n">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>2026-02-23 11:51:13</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650PE</t>
+        </is>
+      </c>
+      <c r="C641" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="D641" t="n">
+        <v>110</v>
+      </c>
+      <c r="E641" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F641" t="n">
+        <v>7280</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>2026-02-23 11:53:43</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C642" t="n">
+        <v>96.55</v>
+      </c>
+      <c r="D642" t="n">
+        <v>103.45</v>
+      </c>
+      <c r="E642" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F642" t="n">
+        <v>8970</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>2026-02-23 11:54:39</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C643" t="n">
+        <v>104.5</v>
+      </c>
+      <c r="D643" t="n">
+        <v>105.85</v>
+      </c>
+      <c r="E643" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F643" t="n">
+        <v>1755</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>2026-02-23 12:11:57</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C644" t="n">
+        <v>102.3</v>
+      </c>
+      <c r="D644" t="n">
+        <v>103.65</v>
+      </c>
+      <c r="E644" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F644" t="n">
+        <v>1755</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>2026-02-23 12:14:12</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25650CE</t>
+        </is>
+      </c>
+      <c r="C645" t="n">
+        <v>108.75</v>
+      </c>
+      <c r="D645" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="E645" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F645" t="n">
+        <v>-12155</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>2026-02-24 10:57:14</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25550PE</t>
+        </is>
+      </c>
+      <c r="C646" t="n">
+        <v>108.9</v>
+      </c>
+      <c r="D646" t="n">
+        <v>110.45</v>
+      </c>
+      <c r="E646" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F646" t="n">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>2026-02-24 10:57:48</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25550PE</t>
+        </is>
+      </c>
+      <c r="C647" t="n">
+        <v>108.55</v>
+      </c>
+      <c r="D647" t="n">
+        <v>109.25</v>
+      </c>
+      <c r="E647" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F647" t="n">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>2026-02-24 10:58:07</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25550PE</t>
+        </is>
+      </c>
+      <c r="C648" t="n">
+        <v>108.95</v>
+      </c>
+      <c r="D648" t="n">
+        <v>109.4</v>
+      </c>
+      <c r="E648" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F648" t="n">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>2026-02-24 11:06:07</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>NIFTY2630225300PE</t>
+        </is>
+      </c>
+      <c r="C649" t="n">
+        <v>105.1</v>
+      </c>
+      <c r="D649" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="E649" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F649" t="n">
+        <v>3510</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>2026-02-24 11:07:22</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25400CE</t>
+        </is>
+      </c>
+      <c r="C650" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="D650" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="E650" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F650" t="n">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>2026-02-24 11:08:48</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>SENSEX26FEB83500CE</t>
+        </is>
+      </c>
+      <c r="C651" t="n">
+        <v>115.8</v>
+      </c>
+      <c r="D651" t="n">
+        <v>117.65</v>
+      </c>
+      <c r="E651" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F651" t="n">
+        <v>1850</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>2026-02-24 11:30:18</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25450CE</t>
+        </is>
+      </c>
+      <c r="C652" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="D652" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="E652" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F652" t="n">
+        <v>975</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>2026-02-24 11:49:06</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25600PE</t>
+        </is>
+      </c>
+      <c r="C653" t="n">
+        <v>119.25</v>
+      </c>
+      <c r="D653" t="n">
+        <v>119.4</v>
+      </c>
+      <c r="E653" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F653" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>2026-02-24 11:51:06</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25600PE</t>
+        </is>
+      </c>
+      <c r="C654" t="n">
+        <v>118.15</v>
+      </c>
+      <c r="D654" t="n">
+        <v>121.2</v>
+      </c>
+      <c r="E654" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F654" t="n">
+        <v>3965</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>2026-02-24 11:56:43</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25600PE</t>
+        </is>
+      </c>
+      <c r="C655" t="n">
+        <v>121.3</v>
+      </c>
+      <c r="D655" t="n">
+        <v>122</v>
+      </c>
+      <c r="E655" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F655" t="n">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>2026-02-24 12:01:14</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25550PE</t>
+        </is>
+      </c>
+      <c r="C656" t="n">
+        <v>99.90000000000001</v>
+      </c>
+      <c r="D656" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="E656" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F656" t="n">
+        <v>2080</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>2026-02-24 12:01:38</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25550PE</t>
+        </is>
+      </c>
+      <c r="C657" t="n">
+        <v>104.15</v>
+      </c>
+      <c r="D657" t="n">
+        <v>105.4</v>
+      </c>
+      <c r="E657" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F657" t="n">
+        <v>1625</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>2026-02-24 12:03:35</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>NIFTY26FEB25550PE</t>
+        </is>
+      </c>
+      <c r="C658" t="n">
+        <v>104.7</v>
+      </c>
+      <c r="D658" t="n">
+        <v>108.05</v>
+      </c>
+      <c r="E658" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F658" t="n">
+        <v>4355</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sync latest changes from main: bot updates, Fibonacci analyzer, AI analysis summaries
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Lakshmi.xlsx
+++ b/Lakshmi.xlsx
@@ -519,7 +519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H920"/>
+  <dimension ref="A1:I931"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="24.33203125" customWidth="1" style="1" min="1" max="1"/>
@@ -25932,6 +25932,341 @@
         <v>3510</v>
       </c>
       <c r="G920" t="inlineStr">
+        <is>
+          <t>PAPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>2026-05-13 12:18:00</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>NIFTY2651923300PE</t>
+        </is>
+      </c>
+      <c r="C921" t="n">
+        <v>140.35</v>
+      </c>
+      <c r="D921" t="n">
+        <v>143.1</v>
+      </c>
+      <c r="E921" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F921" t="n">
+        <v>3575</v>
+      </c>
+      <c r="G921" t="inlineStr">
+        <is>
+          <t>PAPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>2026-05-13 13:29:51</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>NIFTY2651923300PE</t>
+        </is>
+      </c>
+      <c r="C922" t="n">
+        <v>136.5</v>
+      </c>
+      <c r="D922" t="n">
+        <v>137.75</v>
+      </c>
+      <c r="E922" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F922" t="n">
+        <v>1625</v>
+      </c>
+      <c r="G922" t="inlineStr">
+        <is>
+          <t>PAPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>2026-05-13 13:31:35</t>
+        </is>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>NIFTY2651923300PE</t>
+        </is>
+      </c>
+      <c r="C923" t="n">
+        <v>139.65</v>
+      </c>
+      <c r="D923" t="n">
+        <v>131.7</v>
+      </c>
+      <c r="E923" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F923" t="n">
+        <v>-10335</v>
+      </c>
+      <c r="G923" t="inlineStr">
+        <is>
+          <t>PAPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>2026-05-13 13:36:16</t>
+        </is>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>NIFTY2651923700CE</t>
+        </is>
+      </c>
+      <c r="C924" t="n">
+        <v>160</v>
+      </c>
+      <c r="D924" t="n">
+        <v>161.5</v>
+      </c>
+      <c r="E924" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F924" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G924" t="inlineStr">
+        <is>
+          <t>PAPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>2026-05-13 13:39:29</t>
+        </is>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>NIFTY2651923700CE</t>
+        </is>
+      </c>
+      <c r="C925" t="n">
+        <v>159.9</v>
+      </c>
+      <c r="D925" t="n">
+        <v>160.4</v>
+      </c>
+      <c r="E925" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F925" t="n">
+        <v>650</v>
+      </c>
+      <c r="G925" t="inlineStr">
+        <is>
+          <t>PAPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>2026-05-13 13:48:15</t>
+        </is>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>NIFTY2651923700CE</t>
+        </is>
+      </c>
+      <c r="C926" t="n">
+        <v>158.2</v>
+      </c>
+      <c r="D926" t="n">
+        <v>159.3</v>
+      </c>
+      <c r="E926" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F926" t="n">
+        <v>1430</v>
+      </c>
+      <c r="G926" t="inlineStr">
+        <is>
+          <t>PAPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>2026-05-13 13:56:09</t>
+        </is>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>NIFTY2651923300PE</t>
+        </is>
+      </c>
+      <c r="C927" t="n">
+        <v>140.5</v>
+      </c>
+      <c r="D927" t="n">
+        <v>145.2</v>
+      </c>
+      <c r="E927" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F927" t="n">
+        <v>6110</v>
+      </c>
+      <c r="G927" t="inlineStr">
+        <is>
+          <t>PAPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>2026-05-13 13:58:36</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>NIFTY2651923700CE</t>
+        </is>
+      </c>
+      <c r="C928" t="n">
+        <v>148.35</v>
+      </c>
+      <c r="D928" t="n">
+        <v>148.05</v>
+      </c>
+      <c r="E928" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F928" t="n">
+        <v>-390</v>
+      </c>
+      <c r="G928" t="inlineStr">
+        <is>
+          <t>PAPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>2026-05-13 14:02:29</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>NIFTY2651923700CE</t>
+        </is>
+      </c>
+      <c r="C929" t="n">
+        <v>147.75</v>
+      </c>
+      <c r="D929" t="n">
+        <v>141.65</v>
+      </c>
+      <c r="E929" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F929" t="n">
+        <v>-7930</v>
+      </c>
+      <c r="G929" t="inlineStr">
+        <is>
+          <t>PAPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>2026-05-13 14:04:56</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>NIFTY2651923300PE</t>
+        </is>
+      </c>
+      <c r="C930" t="n">
+        <v>137.2</v>
+      </c>
+      <c r="D930" t="n">
+        <v>142.35</v>
+      </c>
+      <c r="E930" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F930" t="n">
+        <v>6695</v>
+      </c>
+      <c r="G930" t="n">
+        <v>178360</v>
+      </c>
+      <c r="H930" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I930" t="inlineStr">
+        <is>
+          <t>PAPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>2026-05-13 14:57:17</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>NIFTY2651923700CE</t>
+        </is>
+      </c>
+      <c r="C931" t="n">
+        <v>134.6</v>
+      </c>
+      <c r="D931" t="n">
+        <v>135.75</v>
+      </c>
+      <c r="E931" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F931" t="n">
+        <v>1495</v>
+      </c>
+      <c r="G931" t="n">
+        <v>174980</v>
+      </c>
+      <c r="H931" t="inlineStr">
+        <is>
+          <t>PROFIT</t>
+        </is>
+      </c>
+      <c r="I931" t="inlineStr">
         <is>
           <t>PAPER</t>
         </is>

</xml_diff>